<commit_message>
Auto: update sent log 2026-10-01
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Arts_and_Culture.xlsx
+++ b/results/auto_Cape_Town_Arts_and_Culture.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="40">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -555,9 +555,6 @@
       <c r="D5" t="s">
         <v>27</v>
       </c>
-      <c r="G5" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -572,9 +569,6 @@
       <c r="D6" t="s">
         <v>28</v>
       </c>
-      <c r="G6" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -589,9 +583,6 @@
       <c r="D7" t="s">
         <v>29</v>
       </c>
-      <c r="G7" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -606,9 +597,6 @@
       <c r="D8" t="s">
         <v>30</v>
       </c>
-      <c r="G8" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -623,9 +611,6 @@
       <c r="D9" t="s">
         <v>31</v>
       </c>
-      <c r="G9" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -640,9 +625,6 @@
       <c r="D10" t="s">
         <v>32</v>
       </c>
-      <c r="G10" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -656,9 +638,6 @@
       </c>
       <c r="D11" t="s">
         <v>33</v>
-      </c>
-      <c r="G11" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:7">

</xml_diff>

<commit_message>
Terminal run all categories morning 2026-10-06-0648
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Arts_and_Culture.xlsx
+++ b/results/auto_Cape_Town_Arts_and_Culture.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="38">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -566,6 +566,9 @@
       <c r="D6" t="s">
         <v>26</v>
       </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">

</xml_diff>